<commit_message>
refined version of the ERD and also the excel jumia_database
</commit_message>
<xml_diff>
--- a/jumia_database.xlsx
+++ b/jumia_database.xlsx
@@ -4,23 +4,24 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6800" firstSheet="1" activeTab="5"/>
+    <workbookView windowWidth="10560" windowHeight="6080" firstSheet="13" activeTab="14"/>
   </bookViews>
   <sheets>
-    <sheet name="BRANCHES" sheetId="1" r:id="rId1"/>
+    <sheet name="COUNTRIES" sheetId="16" r:id="rId1"/>
     <sheet name="STORES" sheetId="2" r:id="rId2"/>
-    <sheet name="DEPARTMENTS" sheetId="5" r:id="rId3"/>
-    <sheet name="EMPLOYEES" sheetId="3" r:id="rId4"/>
-    <sheet name="CUSTOMERS" sheetId="7" r:id="rId5"/>
-    <sheet name="ORDER" sheetId="8" r:id="rId6"/>
-    <sheet name="CATEGORIES" sheetId="10" r:id="rId7"/>
-    <sheet name="ORDER DETAILS" sheetId="9" r:id="rId8"/>
-    <sheet name="ACCOUNTS" sheetId="6" r:id="rId9"/>
-    <sheet name="DELIVERIES" sheetId="12" r:id="rId10"/>
+    <sheet name="BRANCHES" sheetId="1" r:id="rId3"/>
+    <sheet name="DEPARTMENTS" sheetId="5" r:id="rId4"/>
+    <sheet name="EMPLOYEES" sheetId="3" r:id="rId5"/>
+    <sheet name="ACCOUNTS" sheetId="6" r:id="rId6"/>
+    <sheet name="CUSTOMERS" sheetId="7" r:id="rId7"/>
+    <sheet name="ORDER" sheetId="8" r:id="rId8"/>
+    <sheet name="ORDER DETAILS" sheetId="9" r:id="rId9"/>
+    <sheet name="CATEGORIES" sheetId="10" r:id="rId10"/>
     <sheet name="PRODUCTS" sheetId="11" r:id="rId11"/>
-    <sheet name="PICKUP STATION" sheetId="13" r:id="rId12"/>
-    <sheet name="PAYMENTS" sheetId="14" r:id="rId13"/>
-    <sheet name="vendor" sheetId="15" r:id="rId14"/>
+    <sheet name="DELIVERIES" sheetId="12" r:id="rId12"/>
+    <sheet name="PICKUP STATION" sheetId="13" r:id="rId13"/>
+    <sheet name="PAYMENTS" sheetId="14" r:id="rId14"/>
+    <sheet name="vendor" sheetId="15" r:id="rId15"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,64 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="234">
+  <si>
+    <t>country_id</t>
+  </si>
+  <si>
+    <t>location</t>
+  </si>
+  <si>
+    <t>kalanda</t>
+  </si>
+  <si>
+    <t>junctionway</t>
+  </si>
+  <si>
+    <t>CBD</t>
+  </si>
+  <si>
+    <t>livera</t>
+  </si>
+  <si>
+    <t>ujite</t>
+  </si>
+  <si>
+    <t>store_id</t>
+  </si>
+  <si>
+    <t>store_name</t>
+  </si>
+  <si>
+    <t>s-01</t>
+  </si>
+  <si>
+    <t>jumia-abuja</t>
+  </si>
+  <si>
+    <t>s-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> jumia johannesburg</t>
+  </si>
+  <si>
+    <t>s-03</t>
+  </si>
+  <si>
+    <t>jumia nairobi</t>
+  </si>
+  <si>
+    <t>s-04</t>
+  </si>
+  <si>
+    <t>jumia zaire</t>
+  </si>
+  <si>
+    <t>s-05</t>
+  </si>
+  <si>
+    <t>juia kampala</t>
+  </si>
   <si>
     <t>branch_ID</t>
   </si>
@@ -96,63 +154,6 @@
     <t>Zaire</t>
   </si>
   <si>
-    <t>branch_id</t>
-  </si>
-  <si>
-    <t>store_id</t>
-  </si>
-  <si>
-    <t>store_name</t>
-  </si>
-  <si>
-    <t>location</t>
-  </si>
-  <si>
-    <t>s-01</t>
-  </si>
-  <si>
-    <t>jumia-abuja</t>
-  </si>
-  <si>
-    <t>kalanda</t>
-  </si>
-  <si>
-    <t>s-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> jumia johannesburg</t>
-  </si>
-  <si>
-    <t>junctionway</t>
-  </si>
-  <si>
-    <t>s-03</t>
-  </si>
-  <si>
-    <t>jumia nairobi</t>
-  </si>
-  <si>
-    <t>CBD</t>
-  </si>
-  <si>
-    <t>s-04</t>
-  </si>
-  <si>
-    <t>jumia zaire</t>
-  </si>
-  <si>
-    <t>livera</t>
-  </si>
-  <si>
-    <t>s-05</t>
-  </si>
-  <si>
-    <t>juia kampala</t>
-  </si>
-  <si>
-    <t>ujite</t>
-  </si>
-  <si>
     <t>dept_id</t>
   </si>
   <si>
@@ -270,45 +271,135 @@
     <t>user_id</t>
   </si>
   <si>
+    <t>username</t>
+  </si>
+  <si>
+    <t>account type</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>contacts</t>
+  </si>
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t>user-1</t>
+  </si>
+  <si>
+    <t>mercy okello</t>
+  </si>
+  <si>
+    <t>customer</t>
+  </si>
+  <si>
+    <t>117@gmail.com</t>
+  </si>
+  <si>
+    <t>user-2</t>
+  </si>
+  <si>
+    <t>kendy q</t>
+  </si>
+  <si>
+    <t>vendor</t>
+  </si>
+  <si>
+    <t>118@gmail.com</t>
+  </si>
+  <si>
+    <t>user-3</t>
+  </si>
+  <si>
+    <t>sauti sol</t>
+  </si>
+  <si>
+    <t>119@gmail.com</t>
+  </si>
+  <si>
+    <t>user-4</t>
+  </si>
+  <si>
+    <t>toxic</t>
+  </si>
+  <si>
+    <t>120@gmail.com</t>
+  </si>
+  <si>
+    <t>user-5</t>
+  </si>
+  <si>
+    <t>m right</t>
+  </si>
+  <si>
+    <t>121@gmail.com</t>
+  </si>
+  <si>
+    <t>user-6</t>
+  </si>
+  <si>
+    <t>jared manyare</t>
+  </si>
+  <si>
+    <t>122@gmail.com</t>
+  </si>
+  <si>
+    <t>user-7</t>
+  </si>
+  <si>
+    <t>chiti</t>
+  </si>
+  <si>
+    <t>123@gmail.com</t>
+  </si>
+  <si>
+    <t>user-8</t>
+  </si>
+  <si>
+    <t>bahati</t>
+  </si>
+  <si>
+    <t>124@gmail.com</t>
+  </si>
+  <si>
+    <t>user-9</t>
+  </si>
+  <si>
+    <t>diana b</t>
+  </si>
+  <si>
+    <t>125@gmail.com</t>
+  </si>
+  <si>
+    <t>user-10</t>
+  </si>
+  <si>
+    <t>dyana cods</t>
+  </si>
+  <si>
+    <t>126@gmail.com</t>
+  </si>
+  <si>
     <t>customer_id</t>
   </si>
   <si>
-    <t>status</t>
-  </si>
-  <si>
-    <t>user-1</t>
+    <t>adress</t>
   </si>
   <si>
     <t>cu-1</t>
   </si>
   <si>
-    <t>active</t>
-  </si>
-  <si>
-    <t>user-4</t>
-  </si>
-  <si>
     <t>cu-4</t>
   </si>
   <si>
-    <t>user-5</t>
-  </si>
-  <si>
     <t>cu-5</t>
   </si>
   <si>
-    <t>dormant</t>
-  </si>
-  <si>
-    <t>user-6</t>
-  </si>
-  <si>
     <t>cu-6</t>
   </si>
   <si>
-    <t>user-7</t>
-  </si>
-  <si>
     <t>cu-7</t>
   </si>
   <si>
@@ -318,229 +409,217 @@
     <t>order number</t>
   </si>
   <si>
+    <t>timestamp</t>
+  </si>
+  <si>
+    <t>abcde</t>
+  </si>
+  <si>
+    <t>order-1</t>
+  </si>
+  <si>
+    <t>abcdf</t>
+  </si>
+  <si>
+    <t>order-2</t>
+  </si>
+  <si>
+    <t>abcdg</t>
+  </si>
+  <si>
+    <t>order-3</t>
+  </si>
+  <si>
+    <t>abcdh</t>
+  </si>
+  <si>
+    <t>order-4</t>
+  </si>
+  <si>
+    <t>abcdi</t>
+  </si>
+  <si>
+    <t>order-5</t>
+  </si>
+  <si>
+    <t>order_details_id</t>
+  </si>
+  <si>
+    <t>quantity</t>
+  </si>
+  <si>
+    <t>product_id</t>
+  </si>
+  <si>
+    <t>3-pieces</t>
+  </si>
+  <si>
+    <t>prod-1</t>
+  </si>
+  <si>
+    <t>4-pieces</t>
+  </si>
+  <si>
+    <t>prod-2</t>
+  </si>
+  <si>
+    <t>5-pieces</t>
+  </si>
+  <si>
+    <t>prod-3</t>
+  </si>
+  <si>
+    <t>6-pieces</t>
+  </si>
+  <si>
+    <t>prod-4</t>
+  </si>
+  <si>
+    <t>7-pieces</t>
+  </si>
+  <si>
+    <t>prod-5</t>
+  </si>
+  <si>
     <t>category_id</t>
   </si>
   <si>
-    <t>product_id</t>
-  </si>
-  <si>
-    <t>timestamp</t>
-  </si>
-  <si>
-    <t>abcde</t>
-  </si>
-  <si>
-    <t>order-1</t>
+    <t>name</t>
+  </si>
+  <si>
+    <t>description</t>
   </si>
   <si>
     <t>cat-1</t>
   </si>
   <si>
-    <t>prod-1</t>
-  </si>
-  <si>
-    <t>abcdf</t>
-  </si>
-  <si>
-    <t>order-2</t>
+    <t>electronics</t>
   </si>
   <si>
     <t>cat-2</t>
   </si>
   <si>
-    <t>prod-2</t>
-  </si>
-  <si>
-    <t>abcdg</t>
-  </si>
-  <si>
-    <t>order-3</t>
+    <t>shoes</t>
   </si>
   <si>
     <t>cat-3</t>
   </si>
   <si>
-    <t>prod-3</t>
-  </si>
-  <si>
-    <t>abcdh</t>
-  </si>
-  <si>
-    <t>order-4</t>
+    <t>clothes</t>
   </si>
   <si>
     <t>cat-4</t>
   </si>
   <si>
-    <t>prod-4</t>
-  </si>
-  <si>
-    <t>abcdi</t>
-  </si>
-  <si>
-    <t>order-5</t>
+    <t>kitchenware</t>
   </si>
   <si>
     <t>cat-5</t>
   </si>
   <si>
-    <t>prod-5</t>
-  </si>
-  <si>
-    <t>name</t>
-  </si>
-  <si>
-    <t>description</t>
-  </si>
-  <si>
-    <t>electronics</t>
-  </si>
-  <si>
-    <t>shoes</t>
-  </si>
-  <si>
-    <t>clothes</t>
-  </si>
-  <si>
-    <t>kitchenware</t>
-  </si>
-  <si>
     <t>detergents</t>
   </si>
   <si>
-    <t>id</t>
-  </si>
-  <si>
-    <t>quantity</t>
-  </si>
-  <si>
-    <t>3-pieces</t>
-  </si>
-  <si>
-    <t>4-pieces</t>
-  </si>
-  <si>
-    <t>5-pieces</t>
-  </si>
-  <si>
-    <t>6-pieces</t>
-  </si>
-  <si>
-    <t>7-pieces</t>
-  </si>
-  <si>
-    <t>username</t>
-  </si>
-  <si>
-    <t>account type</t>
-  </si>
-  <si>
     <t>vendor_id</t>
   </si>
   <si>
-    <t>email</t>
-  </si>
-  <si>
-    <t>contacts</t>
-  </si>
-  <si>
-    <t>password</t>
-  </si>
-  <si>
-    <t>mercy okello</t>
-  </si>
-  <si>
-    <t>customer</t>
-  </si>
-  <si>
-    <t>117@gmail.com</t>
-  </si>
-  <si>
-    <t>user-2</t>
-  </si>
-  <si>
-    <t>kendy q</t>
-  </si>
-  <si>
-    <t>cu-2</t>
-  </si>
-  <si>
-    <t>vendor</t>
-  </si>
-  <si>
-    <t>118@gmail.com</t>
-  </si>
-  <si>
-    <t>user-3</t>
-  </si>
-  <si>
-    <t>sauti sol</t>
-  </si>
-  <si>
-    <t>cu-3</t>
-  </si>
-  <si>
-    <t>119@gmail.com</t>
-  </si>
-  <si>
-    <t>toxic</t>
-  </si>
-  <si>
-    <t>120@gmail.com</t>
-  </si>
-  <si>
-    <t>m right</t>
-  </si>
-  <si>
-    <t>121@gmail.com</t>
-  </si>
-  <si>
-    <t>jared manyare</t>
-  </si>
-  <si>
-    <t>122@gmail.com</t>
-  </si>
-  <si>
-    <t>chiti</t>
-  </si>
-  <si>
-    <t>123@gmail.com</t>
-  </si>
-  <si>
-    <t>user-8</t>
-  </si>
-  <si>
-    <t>bahati</t>
-  </si>
-  <si>
-    <t>cu-8</t>
-  </si>
-  <si>
-    <t>124@gmail.com</t>
-  </si>
-  <si>
-    <t>user-9</t>
-  </si>
-  <si>
-    <t>diana b</t>
-  </si>
-  <si>
-    <t>cu-9</t>
-  </si>
-  <si>
-    <t>125@gmail.com</t>
-  </si>
-  <si>
-    <t>user-10</t>
-  </si>
-  <si>
-    <t>dyana cods</t>
-  </si>
-  <si>
-    <t>cu-10</t>
-  </si>
-  <si>
-    <t>126@gmail.com</t>
+    <t>price</t>
+  </si>
+  <si>
+    <t>brand</t>
+  </si>
+  <si>
+    <t>vendor-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> tv</t>
+  </si>
+  <si>
+    <t>32' inch</t>
+  </si>
+  <si>
+    <t>52000 sh</t>
+  </si>
+  <si>
+    <t>vitron,samsung</t>
+  </si>
+  <si>
+    <t>vendor-2</t>
+  </si>
+  <si>
+    <t>shoe</t>
+  </si>
+  <si>
+    <t>black leather</t>
+  </si>
+  <si>
+    <t>1500 sh</t>
+  </si>
+  <si>
+    <t>nike,new balance</t>
+  </si>
+  <si>
+    <t>vendor-3</t>
+  </si>
+  <si>
+    <t>shirt</t>
+  </si>
+  <si>
+    <t>3d shirt</t>
+  </si>
+  <si>
+    <t>700 sh</t>
+  </si>
+  <si>
+    <t>chrome arts,dior</t>
+  </si>
+  <si>
+    <t>vendor-4</t>
+  </si>
+  <si>
+    <t>laptop</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> dell x touchpad</t>
+  </si>
+  <si>
+    <t>42000 sh</t>
+  </si>
+  <si>
+    <t>dell.lenovo,HP,apple</t>
+  </si>
+  <si>
+    <t>vendor-5</t>
+  </si>
+  <si>
+    <t>mouse</t>
+  </si>
+  <si>
+    <t>roller mouse</t>
+  </si>
+  <si>
+    <t>10000 sh</t>
+  </si>
+  <si>
+    <t>apple,HP</t>
+  </si>
+  <si>
+    <t>prod-6</t>
+  </si>
+  <si>
+    <t>vendor 4</t>
+  </si>
+  <si>
+    <t>spoons</t>
+  </si>
+  <si>
+    <t>silver</t>
+  </si>
+  <si>
+    <t>300 sh</t>
+  </si>
+  <si>
+    <t>kentra</t>
   </si>
   <si>
     <t>delivery_id</t>
@@ -595,105 +674,6 @@
   </si>
   <si>
     <t>pck-e</t>
-  </si>
-  <si>
-    <t>price</t>
-  </si>
-  <si>
-    <t>brand</t>
-  </si>
-  <si>
-    <t>vendor-1</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> tv</t>
-  </si>
-  <si>
-    <t>32' inch</t>
-  </si>
-  <si>
-    <t>52000 sh</t>
-  </si>
-  <si>
-    <t>vitron,samsung</t>
-  </si>
-  <si>
-    <t>vendor-2</t>
-  </si>
-  <si>
-    <t>shoe</t>
-  </si>
-  <si>
-    <t>black leather</t>
-  </si>
-  <si>
-    <t>1500 sh</t>
-  </si>
-  <si>
-    <t>nike,new balance</t>
-  </si>
-  <si>
-    <t>vendor-3</t>
-  </si>
-  <si>
-    <t>shirt</t>
-  </si>
-  <si>
-    <t>3d shirt</t>
-  </si>
-  <si>
-    <t>700 sh</t>
-  </si>
-  <si>
-    <t>chrome arts,dior</t>
-  </si>
-  <si>
-    <t>vendor-4</t>
-  </si>
-  <si>
-    <t>laptop</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> dell x touchpad</t>
-  </si>
-  <si>
-    <t>42000 sh</t>
-  </si>
-  <si>
-    <t>dell.lenovo,HP,apple</t>
-  </si>
-  <si>
-    <t>vendor-5</t>
-  </si>
-  <si>
-    <t>mouse</t>
-  </si>
-  <si>
-    <t>roller mouse</t>
-  </si>
-  <si>
-    <t>10000 sh</t>
-  </si>
-  <si>
-    <t>apple,HP</t>
-  </si>
-  <si>
-    <t>prod-6</t>
-  </si>
-  <si>
-    <t>vendor 4</t>
-  </si>
-  <si>
-    <t>spoons</t>
-  </si>
-  <si>
-    <t>silver</t>
-  </si>
-  <si>
-    <t>300 sh</t>
-  </si>
-  <si>
-    <t>kentra</t>
   </si>
   <si>
     <t>limuru station</t>
@@ -1383,13 +1363,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
@@ -1931,78 +1911,44 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="5" outlineLevelCol="2"/>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="5" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="10.6363636363636" customWidth="1"/>
-    <col min="2" max="2" width="12.8181818181818" customWidth="1"/>
-    <col min="3" max="3" width="20.1818181818182" customWidth="1"/>
+    <col min="1" max="1" width="12.9090909090909" customWidth="1"/>
+    <col min="2" max="2" width="11.7272727272727" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+    </row>
+    <row r="2" spans="2:2">
+      <c r="B2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
+    <row r="3" spans="2:2">
+      <c r="B3" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="4" spans="2:2">
+      <c r="B4" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
+    </row>
+    <row r="5" spans="2:2">
+      <c r="B5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
+    <row r="6" spans="2:2">
+      <c r="B6" t="s">
         <v>6</v>
-      </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" t="s">
-        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -2014,115 +1960,63 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="5" outlineLevelCol="4"/>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="5" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="13.7272727272727" customWidth="1"/>
-    <col min="2" max="2" width="12.4545454545455" customWidth="1"/>
-    <col min="4" max="4" width="15.1818181818182" customWidth="1"/>
-    <col min="5" max="5" width="15.5454545454545" customWidth="1"/>
+    <col min="1" max="1" width="10.8181818181818" customWidth="1"/>
+    <col min="2" max="2" width="11.4545454545455" customWidth="1"/>
+    <col min="3" max="3" width="11.0909090909091" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>167</v>
+        <v>146</v>
       </c>
       <c r="B1" t="s">
-        <v>90</v>
+        <v>147</v>
       </c>
       <c r="C1" t="s">
-        <v>168</v>
-      </c>
-      <c r="D1" t="s">
-        <v>169</v>
-      </c>
-      <c r="E1" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>171</v>
+        <v>149</v>
       </c>
       <c r="B2" t="s">
-        <v>95</v>
-      </c>
-      <c r="C2" t="s">
-        <v>172</v>
-      </c>
-      <c r="D2" t="s">
-        <v>173</v>
-      </c>
-      <c r="E2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>174</v>
+        <v>151</v>
       </c>
       <c r="B3" t="s">
-        <v>99</v>
-      </c>
-      <c r="C3" t="s">
-        <v>175</v>
-      </c>
-      <c r="D3" t="s">
-        <v>176</v>
-      </c>
-      <c r="E3" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>177</v>
+        <v>153</v>
       </c>
       <c r="B4" t="s">
-        <v>103</v>
-      </c>
-      <c r="C4" t="s">
-        <v>178</v>
-      </c>
-      <c r="D4" t="s">
-        <v>179</v>
-      </c>
-      <c r="E4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>180</v>
+        <v>155</v>
       </c>
       <c r="B5" t="s">
-        <v>107</v>
-      </c>
-      <c r="C5" t="s">
-        <v>181</v>
-      </c>
-      <c r="D5" t="s">
-        <v>182</v>
-      </c>
-      <c r="E5" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>183</v>
+        <v>157</v>
       </c>
       <c r="B6" t="s">
-        <v>111</v>
-      </c>
-      <c r="C6" t="s">
-        <v>184</v>
-      </c>
-      <c r="D6" t="s">
-        <v>182</v>
-      </c>
-      <c r="E6" t="s">
-        <v>59</v>
+        <v>158</v>
       </c>
     </row>
   </sheetData>
@@ -2146,163 +2040,163 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" t="s">
-        <v>93</v>
+        <v>135</v>
       </c>
       <c r="B1" t="s">
-        <v>92</v>
+        <v>146</v>
       </c>
       <c r="C1" t="s">
-        <v>131</v>
+        <v>159</v>
       </c>
       <c r="D1" t="s">
-        <v>115</v>
+        <v>147</v>
       </c>
       <c r="E1" t="s">
-        <v>116</v>
+        <v>148</v>
       </c>
       <c r="F1" t="s">
-        <v>185</v>
+        <v>160</v>
       </c>
       <c r="G1" t="s">
-        <v>186</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>98</v>
+        <v>137</v>
       </c>
       <c r="B2" t="s">
-        <v>97</v>
+        <v>149</v>
       </c>
       <c r="C2" t="s">
-        <v>187</v>
+        <v>162</v>
       </c>
       <c r="D2" t="s">
-        <v>188</v>
+        <v>163</v>
       </c>
       <c r="E2" t="s">
-        <v>189</v>
+        <v>164</v>
       </c>
       <c r="F2" t="s">
-        <v>190</v>
+        <v>165</v>
       </c>
       <c r="G2" t="s">
-        <v>191</v>
+        <v>166</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>102</v>
+        <v>139</v>
       </c>
       <c r="B3" t="s">
-        <v>101</v>
+        <v>151</v>
       </c>
       <c r="C3" t="s">
-        <v>192</v>
+        <v>167</v>
       </c>
       <c r="D3" t="s">
-        <v>193</v>
+        <v>168</v>
       </c>
       <c r="E3" t="s">
-        <v>194</v>
+        <v>169</v>
       </c>
       <c r="F3" t="s">
-        <v>195</v>
+        <v>170</v>
       </c>
       <c r="G3" t="s">
-        <v>196</v>
+        <v>171</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>106</v>
+        <v>141</v>
       </c>
       <c r="B4" t="s">
-        <v>105</v>
+        <v>153</v>
       </c>
       <c r="C4" t="s">
-        <v>197</v>
+        <v>172</v>
       </c>
       <c r="D4" t="s">
-        <v>198</v>
+        <v>173</v>
       </c>
       <c r="E4" t="s">
-        <v>199</v>
+        <v>174</v>
       </c>
       <c r="F4" t="s">
-        <v>200</v>
+        <v>175</v>
       </c>
       <c r="G4" t="s">
-        <v>201</v>
+        <v>176</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>110</v>
+        <v>143</v>
       </c>
       <c r="B5" t="s">
-        <v>97</v>
+        <v>149</v>
       </c>
       <c r="C5" t="s">
-        <v>202</v>
+        <v>177</v>
       </c>
       <c r="D5" t="s">
-        <v>203</v>
+        <v>178</v>
       </c>
       <c r="E5" t="s">
-        <v>204</v>
+        <v>179</v>
       </c>
       <c r="F5" t="s">
-        <v>205</v>
+        <v>180</v>
       </c>
       <c r="G5" t="s">
-        <v>206</v>
+        <v>181</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>114</v>
+        <v>145</v>
       </c>
       <c r="B6" t="s">
-        <v>97</v>
+        <v>149</v>
       </c>
       <c r="C6" t="s">
-        <v>207</v>
+        <v>182</v>
       </c>
       <c r="D6" t="s">
-        <v>208</v>
+        <v>183</v>
       </c>
       <c r="E6" t="s">
-        <v>209</v>
+        <v>184</v>
       </c>
       <c r="F6" t="s">
-        <v>210</v>
+        <v>185</v>
       </c>
       <c r="G6" t="s">
-        <v>211</v>
+        <v>186</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>212</v>
+        <v>187</v>
       </c>
       <c r="B7" t="s">
-        <v>109</v>
+        <v>155</v>
       </c>
       <c r="C7" t="s">
-        <v>213</v>
+        <v>188</v>
       </c>
       <c r="D7" t="s">
-        <v>214</v>
+        <v>189</v>
       </c>
       <c r="E7" t="s">
-        <v>215</v>
+        <v>190</v>
       </c>
       <c r="F7" t="s">
-        <v>216</v>
+        <v>191</v>
       </c>
       <c r="G7" t="s">
-        <v>217</v>
+        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -2312,6 +2206,126 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="5" outlineLevelCol="4"/>
+  <cols>
+    <col min="1" max="1" width="13.7272727272727" customWidth="1"/>
+    <col min="2" max="2" width="12.4545454545455" customWidth="1"/>
+    <col min="4" max="4" width="15.1818181818182" customWidth="1"/>
+    <col min="5" max="5" width="15.5454545454545" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>193</v>
+      </c>
+      <c r="B1" t="s">
+        <v>120</v>
+      </c>
+      <c r="C1" t="s">
+        <v>194</v>
+      </c>
+      <c r="D1" t="s">
+        <v>195</v>
+      </c>
+      <c r="E1" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>197</v>
+      </c>
+      <c r="B2" t="s">
+        <v>123</v>
+      </c>
+      <c r="C2" t="s">
+        <v>198</v>
+      </c>
+      <c r="D2" t="s">
+        <v>199</v>
+      </c>
+      <c r="E2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>200</v>
+      </c>
+      <c r="B3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C3" t="s">
+        <v>201</v>
+      </c>
+      <c r="D3" t="s">
+        <v>202</v>
+      </c>
+      <c r="E3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B4" t="s">
+        <v>127</v>
+      </c>
+      <c r="C4" t="s">
+        <v>204</v>
+      </c>
+      <c r="D4" t="s">
+        <v>205</v>
+      </c>
+      <c r="E4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>206</v>
+      </c>
+      <c r="B5" t="s">
+        <v>129</v>
+      </c>
+      <c r="C5" t="s">
+        <v>207</v>
+      </c>
+      <c r="D5" t="s">
+        <v>208</v>
+      </c>
+      <c r="E5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>209</v>
+      </c>
+      <c r="B6" t="s">
+        <v>131</v>
+      </c>
+      <c r="C6" t="s">
+        <v>210</v>
+      </c>
+      <c r="D6" t="s">
+        <v>208</v>
+      </c>
+      <c r="E6" t="s">
+        <v>59</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:C6"/>
@@ -2322,68 +2336,68 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>168</v>
+        <v>194</v>
       </c>
       <c r="B1" t="s">
-        <v>115</v>
+        <v>147</v>
       </c>
       <c r="C1" t="s">
-        <v>115</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>172</v>
+        <v>198</v>
       </c>
       <c r="B2" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="C2" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>175</v>
+        <v>201</v>
       </c>
       <c r="B3" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="C3" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>178</v>
+        <v>204</v>
       </c>
       <c r="B4" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="C4" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>181</v>
+        <v>207</v>
       </c>
       <c r="B5" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="C5" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>184</v>
+        <v>210</v>
       </c>
       <c r="B6" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="C6" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
     </row>
   </sheetData>
@@ -2392,7 +2406,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:D6"/>
@@ -2406,86 +2420,86 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="B1" t="s">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="C1" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="D1" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="B2" t="s">
-        <v>95</v>
+        <v>123</v>
       </c>
       <c r="C2" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="D2" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="B3" t="s">
-        <v>99</v>
+        <v>125</v>
       </c>
       <c r="C3" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="D3" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="B4" t="s">
-        <v>103</v>
+        <v>127</v>
       </c>
       <c r="C4" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="D4" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="B5" t="s">
-        <v>107</v>
+        <v>129</v>
       </c>
       <c r="C5" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="D5" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="B6" t="s">
-        <v>111</v>
+        <v>131</v>
       </c>
       <c r="C6" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="D6" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
     </row>
   </sheetData>
@@ -2494,7 +2508,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:D6"/>
@@ -2505,13 +2519,13 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>131</v>
+        <v>159</v>
       </c>
       <c r="B1" t="s">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="C1" t="s">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="D1" t="s">
         <v>75</v>
@@ -2519,72 +2533,72 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>187</v>
+        <v>162</v>
       </c>
       <c r="B2" t="s">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="D2" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>192</v>
+        <v>167</v>
       </c>
       <c r="B3" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>27</v>
+        <v>3</v>
       </c>
       <c r="D3" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>197</v>
+        <v>172</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="D4" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>202</v>
+        <v>177</v>
       </c>
       <c r="B5" t="s">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="C5" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="D5" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>207</v>
+        <v>182</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>6</v>
       </c>
       <c r="D6" t="s">
-        <v>163</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -2599,92 +2613,77 @@
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="5" outlineLevelCol="3"/>
   <cols>
-    <col min="3" max="3" width="20.9090909090909" customWidth="1"/>
+    <col min="2" max="3" width="20.9090909090909" customWidth="1"/>
     <col min="4" max="4" width="11.7272727272727" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="B1" t="s">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="D1" t="s">
-        <v>21</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="D2" t="s">
-        <v>24</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>27</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
         <v>15</v>
       </c>
-      <c r="B5" t="s">
-        <v>31</v>
-      </c>
       <c r="C5" t="s">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="D5" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="D6" t="s">
-        <v>36</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -2699,8 +2698,9 @@
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="5" outlineLevelCol="3"/>
   <cols>
-    <col min="2" max="3" width="10.6363636363636" customWidth="1"/>
-    <col min="4" max="4" width="14.9090909090909" customWidth="1"/>
+    <col min="1" max="1" width="10.6363636363636" customWidth="1"/>
+    <col min="3" max="3" width="12.8181818181818" customWidth="1"/>
+    <col min="4" max="4" width="20.1818181818182" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -2708,13 +2708,13 @@
         <v>19</v>
       </c>
       <c r="B1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C1" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="D1" t="s">
-        <v>38</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -2722,13 +2722,13 @@
         <v>22</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="D2" t="s">
-        <v>40</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -2736,13 +2736,13 @@
         <v>25</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="D3" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -2750,13 +2750,13 @@
         <v>28</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="D4" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -2764,13 +2764,13 @@
         <v>31</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C5" t="s">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="D5" t="s">
-        <v>46</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -2778,13 +2778,13 @@
         <v>34</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -2794,6 +2794,88 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="5" outlineLevelCol="2"/>
+  <cols>
+    <col min="1" max="2" width="10.6363636363636" customWidth="1"/>
+    <col min="3" max="3" width="14.9090909090909" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G6"/>
@@ -2939,223 +3021,250 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="5" outlineLevelCol="2"/>
-  <cols>
-    <col min="2" max="2" width="11.2727272727273" customWidth="1"/>
-    <col min="3" max="3" width="16.0909090909091" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>75</v>
-      </c>
-      <c r="B1" t="s">
-        <v>76</v>
-      </c>
-      <c r="C1" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>78</v>
-      </c>
-      <c r="B2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C2" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>81</v>
-      </c>
-      <c r="B3" t="s">
-        <v>82</v>
-      </c>
-      <c r="C3" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
-        <v>83</v>
-      </c>
-      <c r="B4" t="s">
-        <v>84</v>
-      </c>
-      <c r="C4" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
-        <v>86</v>
-      </c>
-      <c r="B5" t="s">
-        <v>87</v>
-      </c>
-      <c r="C5" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
-        <v>88</v>
-      </c>
-      <c r="B6" t="s">
-        <v>89</v>
-      </c>
-      <c r="C6" t="s">
-        <v>80</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="5" outlineLevelCol="5"/>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="12.4545454545455" customWidth="1"/>
-    <col min="2" max="2" width="16.0909090909091" customWidth="1"/>
-    <col min="3" max="3" width="10.8181818181818" customWidth="1"/>
-    <col min="4" max="4" width="9.81818181818182" customWidth="1"/>
-    <col min="5" max="5" width="11.2727272727273" customWidth="1"/>
-    <col min="6" max="6" width="9.45454545454546"/>
+    <col min="2" max="2" width="13.6363636363636" customWidth="1"/>
+    <col min="3" max="3" width="13.0909090909091" customWidth="1"/>
+    <col min="4" max="4" width="17.3636363636364" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="B1" t="s">
-        <v>91</v>
+        <v>76</v>
       </c>
       <c r="C1" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="D1" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="E1" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="F1" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="B2" t="s">
-        <v>96</v>
+        <v>82</v>
       </c>
       <c r="C2" t="s">
-        <v>97</v>
-      </c>
-      <c r="D2" t="s">
-        <v>98</v>
-      </c>
-      <c r="E2" t="s">
-        <v>79</v>
-      </c>
-      <c r="F2" s="3">
-        <v>0.396527777777778</v>
+        <v>83</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E2">
+        <v>8150</v>
+      </c>
+      <c r="F2">
+        <v>12347</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>99</v>
+        <v>85</v>
       </c>
       <c r="B3" t="s">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="C3" t="s">
-        <v>101</v>
-      </c>
-      <c r="D3" t="s">
-        <v>102</v>
-      </c>
-      <c r="E3" t="s">
-        <v>82</v>
-      </c>
-      <c r="F3" s="3">
-        <v>0.438194444444444</v>
+        <v>87</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="E3">
+        <v>8151</v>
+      </c>
+      <c r="F3">
+        <v>12348</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>103</v>
+        <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>104</v>
+        <v>90</v>
       </c>
       <c r="C4" t="s">
-        <v>105</v>
-      </c>
-      <c r="D4" t="s">
-        <v>106</v>
-      </c>
-      <c r="E4" t="s">
-        <v>84</v>
-      </c>
-      <c r="F4" s="3">
-        <v>0.479861111111111</v>
+        <v>87</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E4">
+        <v>8152</v>
+      </c>
+      <c r="F4">
+        <v>12349</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>107</v>
+        <v>92</v>
       </c>
       <c r="B5" t="s">
-        <v>108</v>
+        <v>93</v>
       </c>
       <c r="C5" t="s">
-        <v>109</v>
-      </c>
-      <c r="D5" t="s">
-        <v>110</v>
-      </c>
-      <c r="E5" t="s">
-        <v>87</v>
-      </c>
-      <c r="F5" s="3">
-        <v>0.521527777777778</v>
+        <v>83</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="E5">
+        <v>8153</v>
+      </c>
+      <c r="F5">
+        <v>12350</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
+        <v>95</v>
+      </c>
+      <c r="B6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C6" t="s">
+        <v>83</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E6">
+        <v>8154</v>
+      </c>
+      <c r="F6">
+        <v>12351</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" t="s">
+        <v>98</v>
+      </c>
+      <c r="B7" t="s">
+        <v>99</v>
+      </c>
+      <c r="C7" t="s">
+        <v>83</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="E7">
+        <v>8155</v>
+      </c>
+      <c r="F7">
+        <v>12352</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" t="s">
+        <v>101</v>
+      </c>
+      <c r="B8" t="s">
+        <v>102</v>
+      </c>
+      <c r="C8" t="s">
+        <v>83</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="E8">
+        <v>8156</v>
+      </c>
+      <c r="F8">
+        <v>12353</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" t="s">
+        <v>104</v>
+      </c>
+      <c r="B9" t="s">
+        <v>105</v>
+      </c>
+      <c r="C9" t="s">
+        <v>87</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="E9">
+        <v>8157</v>
+      </c>
+      <c r="F9">
+        <v>12354</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" t="s">
+        <v>107</v>
+      </c>
+      <c r="B10" t="s">
+        <v>108</v>
+      </c>
+      <c r="C10" t="s">
+        <v>87</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="E10">
+        <v>8158</v>
+      </c>
+      <c r="F10">
+        <v>12355</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" t="s">
+        <v>110</v>
+      </c>
+      <c r="B11" t="s">
         <v>111</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C11" t="s">
+        <v>87</v>
+      </c>
+      <c r="D11" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="C6" t="s">
-        <v>113</v>
-      </c>
-      <c r="D6" t="s">
-        <v>114</v>
-      </c>
-      <c r="E6" t="s">
-        <v>89</v>
-      </c>
-      <c r="F6" s="3">
-        <v>0.563194444444444</v>
+      <c r="E11">
+        <v>8159</v>
+      </c>
+      <c r="F11">
+        <v>12356</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D3" r:id="rId1" display="118@gmail.com"/>
+    <hyperlink ref="D4" r:id="rId1" display="119@gmail.com"/>
+    <hyperlink ref="D5" r:id="rId1" display="120@gmail.com"/>
+    <hyperlink ref="D6" r:id="rId1" display="121@gmail.com"/>
+    <hyperlink ref="D2" r:id="rId2" display="117@gmail.com"/>
+    <hyperlink ref="D7" r:id="rId1" display="122@gmail.com"/>
+    <hyperlink ref="D8" r:id="rId1" display="123@gmail.com"/>
+    <hyperlink ref="D9" r:id="rId1" display="124@gmail.com"/>
+    <hyperlink ref="D10" r:id="rId1" display="125@gmail.com"/>
+    <hyperlink ref="D11" r:id="rId1" display="126@gmail.com"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
@@ -3167,60 +3276,58 @@
   <dimension ref="A1:C6"/>
   <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="5" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="10.8181818181818" customWidth="1"/>
-    <col min="2" max="2" width="11.4545454545455" customWidth="1"/>
-    <col min="3" max="3" width="11.0909090909091" customWidth="1"/>
+    <col min="2" max="2" width="11.2727272727273" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>92</v>
+        <v>75</v>
       </c>
       <c r="B1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="B2" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="B3" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="B4" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="B5" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="B6" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -3236,92 +3343,93 @@
   <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="5" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="12.4545454545455" customWidth="1"/>
-    <col min="2" max="2" width="11.2727272727273" customWidth="1"/>
-    <col min="4" max="4" width="9.81818181818182" customWidth="1"/>
+    <col min="2" max="2" width="16.0909090909091" customWidth="1"/>
+    <col min="3" max="3" width="11.2727272727273" customWidth="1"/>
+    <col min="4" max="4" width="9.45454545454546"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="B1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C1" t="s">
+        <v>113</v>
+      </c>
+      <c r="D1" t="s">
         <v>122</v>
-      </c>
-      <c r="C1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D1" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>95</v>
-      </c>
-      <c r="B2">
-        <v>10</v>
+        <v>123</v>
+      </c>
+      <c r="B2" t="s">
+        <v>124</v>
       </c>
       <c r="C2" t="s">
-        <v>124</v>
-      </c>
-      <c r="D2" t="s">
-        <v>98</v>
+        <v>115</v>
+      </c>
+      <c r="D2" s="1">
+        <v>0.396527777777778</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>99</v>
-      </c>
-      <c r="B3">
-        <v>11</v>
+        <v>125</v>
+      </c>
+      <c r="B3" t="s">
+        <v>126</v>
       </c>
       <c r="C3" t="s">
-        <v>125</v>
-      </c>
-      <c r="D3" t="s">
-        <v>102</v>
+        <v>116</v>
+      </c>
+      <c r="D3" s="1">
+        <v>0.438194444444444</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>103</v>
-      </c>
-      <c r="B4">
-        <v>12</v>
+        <v>127</v>
+      </c>
+      <c r="B4" t="s">
+        <v>128</v>
       </c>
       <c r="C4" t="s">
-        <v>126</v>
-      </c>
-      <c r="D4" t="s">
-        <v>106</v>
+        <v>117</v>
+      </c>
+      <c r="D4" s="1">
+        <v>0.479861111111111</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>107</v>
-      </c>
-      <c r="B5">
-        <v>13</v>
+        <v>129</v>
+      </c>
+      <c r="B5" t="s">
+        <v>130</v>
       </c>
       <c r="C5" t="s">
-        <v>127</v>
-      </c>
-      <c r="D5" t="s">
-        <v>110</v>
+        <v>118</v>
+      </c>
+      <c r="D5" s="1">
+        <v>0.521527777777778</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>111</v>
-      </c>
-      <c r="B6">
-        <v>14</v>
+        <v>131</v>
+      </c>
+      <c r="B6" t="s">
+        <v>132</v>
       </c>
       <c r="C6" t="s">
-        <v>128</v>
-      </c>
-      <c r="D6" t="s">
-        <v>114</v>
+        <v>119</v>
+      </c>
+      <c r="D6" s="1">
+        <v>0.563194444444444</v>
       </c>
     </row>
   </sheetData>
@@ -3333,318 +3441,99 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:I11"/>
-  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5"/>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="5" outlineLevelCol="3"/>
   <cols>
-    <col min="1" max="1" width="10.6363636363636" customWidth="1"/>
-    <col min="3" max="3" width="13.6363636363636" customWidth="1"/>
-    <col min="4" max="4" width="11.2727272727273" customWidth="1"/>
-    <col min="5" max="5" width="13.0909090909091" customWidth="1"/>
-    <col min="7" max="7" width="17.3636363636364" customWidth="1"/>
+    <col min="1" max="1" width="12.4545454545455" customWidth="1"/>
+    <col min="2" max="2" width="15.9090909090909" customWidth="1"/>
+    <col min="4" max="4" width="9.81818181818182" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="B1" t="s">
-        <v>75</v>
+        <v>133</v>
       </c>
       <c r="C1" t="s">
+        <v>134</v>
+      </c>
+      <c r="D1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B2">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>136</v>
+      </c>
+      <c r="D2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B3">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
+        <v>138</v>
+      </c>
+      <c r="D3" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B4">
+        <v>12</v>
+      </c>
+      <c r="C4" t="s">
+        <v>140</v>
+      </c>
+      <c r="D4" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
         <v>129</v>
       </c>
-      <c r="D1" t="s">
-        <v>76</v>
-      </c>
-      <c r="E1" t="s">
-        <v>130</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="B5">
+        <v>13</v>
+      </c>
+      <c r="C5" t="s">
+        <v>142</v>
+      </c>
+      <c r="D5" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" t="s">
         <v>131</v>
       </c>
-      <c r="G1" t="s">
-        <v>132</v>
-      </c>
-      <c r="H1" t="s">
-        <v>133</v>
-      </c>
-      <c r="I1" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C2" t="s">
-        <v>135</v>
-      </c>
-      <c r="D2" t="s">
-        <v>79</v>
-      </c>
-      <c r="E2" t="s">
-        <v>136</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="H2">
-        <v>8150</v>
-      </c>
-      <c r="I2">
-        <v>12347</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9">
-      <c r="A3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" t="s">
-        <v>138</v>
-      </c>
-      <c r="C3" t="s">
-        <v>139</v>
-      </c>
-      <c r="D3" t="s">
-        <v>140</v>
-      </c>
-      <c r="E3" t="s">
-        <v>141</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="H3">
-        <v>8151</v>
-      </c>
-      <c r="I3">
-        <v>12348</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>143</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="B6">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
         <v>144</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D6" t="s">
         <v>145</v>
       </c>
-      <c r="E4" t="s">
-        <v>141</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="H4">
-        <v>8152</v>
-      </c>
-      <c r="I4">
-        <v>12349</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9">
-      <c r="A5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" t="s">
-        <v>81</v>
-      </c>
-      <c r="C5" t="s">
-        <v>147</v>
-      </c>
-      <c r="D5" t="s">
-        <v>82</v>
-      </c>
-      <c r="E5" t="s">
-        <v>136</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="H5">
-        <v>8153</v>
-      </c>
-      <c r="I5">
-        <v>12350</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9">
-      <c r="A6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" t="s">
-        <v>83</v>
-      </c>
-      <c r="C6" t="s">
-        <v>149</v>
-      </c>
-      <c r="D6" t="s">
-        <v>84</v>
-      </c>
-      <c r="E6" t="s">
-        <v>136</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="H6">
-        <v>8154</v>
-      </c>
-      <c r="I6">
-        <v>12351</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" t="s">
-        <v>86</v>
-      </c>
-      <c r="C7" t="s">
-        <v>151</v>
-      </c>
-      <c r="D7" t="s">
-        <v>87</v>
-      </c>
-      <c r="E7" t="s">
-        <v>136</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="H7">
-        <v>8155</v>
-      </c>
-      <c r="I7">
-        <v>12352</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9">
-      <c r="A8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" t="s">
-        <v>88</v>
-      </c>
-      <c r="C8" t="s">
-        <v>153</v>
-      </c>
-      <c r="D8" t="s">
-        <v>89</v>
-      </c>
-      <c r="E8" t="s">
-        <v>136</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="H8">
-        <v>8156</v>
-      </c>
-      <c r="I8">
-        <v>12353</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9">
-      <c r="A9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" t="s">
-        <v>155</v>
-      </c>
-      <c r="C9" t="s">
-        <v>156</v>
-      </c>
-      <c r="D9" t="s">
-        <v>157</v>
-      </c>
-      <c r="E9" t="s">
-        <v>141</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="H9">
-        <v>8157</v>
-      </c>
-      <c r="I9">
-        <v>12354</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9">
-      <c r="A10" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" t="s">
-        <v>159</v>
-      </c>
-      <c r="C10" t="s">
-        <v>160</v>
-      </c>
-      <c r="D10" t="s">
-        <v>161</v>
-      </c>
-      <c r="E10" t="s">
-        <v>141</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="H10">
-        <v>8158</v>
-      </c>
-      <c r="I10">
-        <v>12355</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9">
-      <c r="A11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" t="s">
-        <v>163</v>
-      </c>
-      <c r="C11" t="s">
-        <v>164</v>
-      </c>
-      <c r="D11" t="s">
-        <v>165</v>
-      </c>
-      <c r="E11" t="s">
-        <v>141</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="H11">
-        <v>8159</v>
-      </c>
-      <c r="I11">
-        <v>12356</v>
-      </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="G3" r:id="rId1" display="118@gmail.com"/>
-    <hyperlink ref="G4" r:id="rId1" display="119@gmail.com"/>
-    <hyperlink ref="G5" r:id="rId1" display="120@gmail.com"/>
-    <hyperlink ref="G6" r:id="rId1" display="121@gmail.com"/>
-    <hyperlink ref="G2" r:id="rId2" display="117@gmail.com"/>
-    <hyperlink ref="G7" r:id="rId1" display="122@gmail.com"/>
-    <hyperlink ref="G8" r:id="rId1" display="123@gmail.com"/>
-    <hyperlink ref="G9" r:id="rId1" display="124@gmail.com"/>
-    <hyperlink ref="G10" r:id="rId1" display="125@gmail.com"/>
-    <hyperlink ref="G11" r:id="rId1" display="126@gmail.com"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>

</xml_diff>

<commit_message>
refined version 3 of the ERD whereby i added a vendor list table to help in maintaining consistence of the data
</commit_message>
<xml_diff>
--- a/jumia_database.xlsx
+++ b/jumia_database.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="10560" windowHeight="6080" firstSheet="13" activeTab="14"/>
+    <workbookView windowWidth="10230" windowHeight="6880" firstSheet="8" activeTab="9"/>
   </bookViews>
   <sheets>
     <sheet name="COUNTRIES" sheetId="16" r:id="rId1"/>
@@ -16,12 +16,13 @@
     <sheet name="CUSTOMERS" sheetId="7" r:id="rId7"/>
     <sheet name="ORDER" sheetId="8" r:id="rId8"/>
     <sheet name="ORDER DETAILS" sheetId="9" r:id="rId9"/>
-    <sheet name="CATEGORIES" sheetId="10" r:id="rId10"/>
-    <sheet name="PRODUCTS" sheetId="11" r:id="rId11"/>
-    <sheet name="DELIVERIES" sheetId="12" r:id="rId12"/>
-    <sheet name="PICKUP STATION" sheetId="13" r:id="rId13"/>
-    <sheet name="PAYMENTS" sheetId="14" r:id="rId14"/>
-    <sheet name="vendor" sheetId="15" r:id="rId15"/>
+    <sheet name="VENDOR LIST" sheetId="17" r:id="rId10"/>
+    <sheet name="CATEGORIES" sheetId="10" r:id="rId11"/>
+    <sheet name="PRODUCTS" sheetId="11" r:id="rId12"/>
+    <sheet name="DELIVERIES" sheetId="12" r:id="rId13"/>
+    <sheet name="PICKUP STATION" sheetId="13" r:id="rId14"/>
+    <sheet name="PAYMENTS" sheetId="14" r:id="rId15"/>
+    <sheet name="vendor" sheetId="15" r:id="rId16"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="231">
   <si>
     <t>country_id</t>
   </si>
@@ -448,301 +449,292 @@
     <t>quantity</t>
   </si>
   <si>
+    <t>listing_id</t>
+  </si>
+  <si>
+    <t>unit_price</t>
+  </si>
+  <si>
+    <t>total</t>
+  </si>
+  <si>
+    <t>3-pieces</t>
+  </si>
+  <si>
+    <t>4-pieces</t>
+  </si>
+  <si>
+    <t>5-pieces</t>
+  </si>
+  <si>
+    <t>6-pieces</t>
+  </si>
+  <si>
+    <t>7-pieces</t>
+  </si>
+  <si>
+    <t>vendor_id</t>
+  </si>
+  <si>
     <t>product_id</t>
   </si>
   <si>
-    <t>3-pieces</t>
+    <t>price</t>
+  </si>
+  <si>
+    <t>stock</t>
+  </si>
+  <si>
+    <t>category_id</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>cat-1</t>
+  </si>
+  <si>
+    <t>electronics</t>
+  </si>
+  <si>
+    <t>cat-2</t>
+  </si>
+  <si>
+    <t>shoes</t>
+  </si>
+  <si>
+    <t>cat-3</t>
+  </si>
+  <si>
+    <t>clothes</t>
+  </si>
+  <si>
+    <t>cat-4</t>
+  </si>
+  <si>
+    <t>kitchenware</t>
+  </si>
+  <si>
+    <t>cat-5</t>
+  </si>
+  <si>
+    <t>detergents</t>
+  </si>
+  <si>
+    <t>brand</t>
   </si>
   <si>
     <t>prod-1</t>
   </si>
   <si>
-    <t>4-pieces</t>
+    <t xml:space="preserve"> tv</t>
+  </si>
+  <si>
+    <t>32' inch</t>
+  </si>
+  <si>
+    <t>vitron</t>
   </si>
   <si>
     <t>prod-2</t>
   </si>
   <si>
-    <t>5-pieces</t>
+    <t>shoe</t>
+  </si>
+  <si>
+    <t>black leather</t>
+  </si>
+  <si>
+    <t>nike</t>
   </si>
   <si>
     <t>prod-3</t>
   </si>
   <si>
-    <t>6-pieces</t>
+    <t>shirt</t>
+  </si>
+  <si>
+    <t>3d shirt</t>
+  </si>
+  <si>
+    <t>chrome</t>
   </si>
   <si>
     <t>prod-4</t>
   </si>
   <si>
-    <t>7-pieces</t>
+    <t>laptop</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> dell x touchpad</t>
+  </si>
+  <si>
+    <t>dell</t>
   </si>
   <si>
     <t>prod-5</t>
   </si>
   <si>
-    <t>category_id</t>
-  </si>
-  <si>
-    <t>name</t>
-  </si>
-  <si>
-    <t>description</t>
-  </si>
-  <si>
-    <t>cat-1</t>
-  </si>
-  <si>
-    <t>electronics</t>
-  </si>
-  <si>
-    <t>cat-2</t>
-  </si>
-  <si>
-    <t>shoes</t>
-  </si>
-  <si>
-    <t>cat-3</t>
-  </si>
-  <si>
-    <t>clothes</t>
-  </si>
-  <si>
-    <t>cat-4</t>
-  </si>
-  <si>
-    <t>kitchenware</t>
-  </si>
-  <si>
-    <t>cat-5</t>
-  </si>
-  <si>
-    <t>detergents</t>
-  </si>
-  <si>
-    <t>vendor_id</t>
-  </si>
-  <si>
-    <t>price</t>
-  </si>
-  <si>
-    <t>brand</t>
+    <t>mouse</t>
+  </si>
+  <si>
+    <t>roller mouse</t>
+  </si>
+  <si>
+    <t>apple</t>
+  </si>
+  <si>
+    <t>prod-6</t>
+  </si>
+  <si>
+    <t>spoons</t>
+  </si>
+  <si>
+    <t>silver</t>
+  </si>
+  <si>
+    <t>kentra</t>
+  </si>
+  <si>
+    <t>delivery_id</t>
+  </si>
+  <si>
+    <t>pck_id</t>
+  </si>
+  <si>
+    <t>delivery_status</t>
+  </si>
+  <si>
+    <t>employee_id</t>
+  </si>
+  <si>
+    <t>delivery-1</t>
+  </si>
+  <si>
+    <t>pck-a</t>
+  </si>
+  <si>
+    <t>shipped</t>
+  </si>
+  <si>
+    <t>delivery-2</t>
+  </si>
+  <si>
+    <t>pck-b</t>
+  </si>
+  <si>
+    <t>in transit</t>
+  </si>
+  <si>
+    <t>delivery-3</t>
+  </si>
+  <si>
+    <t>pck-c</t>
+  </si>
+  <si>
+    <t>in-transit</t>
+  </si>
+  <si>
+    <t>delivery-4</t>
+  </si>
+  <si>
+    <t>pck-d</t>
+  </si>
+  <si>
+    <t>station</t>
+  </si>
+  <si>
+    <t>delivery-5</t>
+  </si>
+  <si>
+    <t>pck-e</t>
+  </si>
+  <si>
+    <t>limuru station</t>
+  </si>
+  <si>
+    <t>limuru</t>
+  </si>
+  <si>
+    <t>nairobi</t>
+  </si>
+  <si>
+    <t>mombasa</t>
+  </si>
+  <si>
+    <t>kisumu</t>
+  </si>
+  <si>
+    <t>machakos</t>
+  </si>
+  <si>
+    <t>payment_id</t>
+  </si>
+  <si>
+    <t>payment method</t>
+  </si>
+  <si>
+    <t>payment status</t>
+  </si>
+  <si>
+    <t>payment-1</t>
+  </si>
+  <si>
+    <t>m-pesa</t>
+  </si>
+  <si>
+    <t>partial</t>
+  </si>
+  <si>
+    <t>payment-2</t>
+  </si>
+  <si>
+    <t>card</t>
+  </si>
+  <si>
+    <t>payment-3</t>
+  </si>
+  <si>
+    <t>mpesa</t>
+  </si>
+  <si>
+    <t>full</t>
+  </si>
+  <si>
+    <t>payment-4</t>
+  </si>
+  <si>
+    <t>payment-5</t>
   </si>
   <si>
     <t>vendor-1</t>
   </si>
   <si>
-    <t xml:space="preserve"> tv</t>
-  </si>
-  <si>
-    <t>32' inch</t>
-  </si>
-  <si>
-    <t>52000 sh</t>
-  </si>
-  <si>
-    <t>vitron,samsung</t>
+    <t>user-02</t>
   </si>
   <si>
     <t>vendor-2</t>
   </si>
   <si>
-    <t>shoe</t>
-  </si>
-  <si>
-    <t>black leather</t>
-  </si>
-  <si>
-    <t>1500 sh</t>
-  </si>
-  <si>
-    <t>nike,new balance</t>
+    <t>user-03</t>
   </si>
   <si>
     <t>vendor-3</t>
   </si>
   <si>
-    <t>shirt</t>
-  </si>
-  <si>
-    <t>3d shirt</t>
-  </si>
-  <si>
-    <t>700 sh</t>
-  </si>
-  <si>
-    <t>chrome arts,dior</t>
+    <t>user-08</t>
   </si>
   <si>
     <t>vendor-4</t>
   </si>
   <si>
-    <t>laptop</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> dell x touchpad</t>
-  </si>
-  <si>
-    <t>42000 sh</t>
-  </si>
-  <si>
-    <t>dell.lenovo,HP,apple</t>
+    <t>user-09</t>
   </si>
   <si>
     <t>vendor-5</t>
-  </si>
-  <si>
-    <t>mouse</t>
-  </si>
-  <si>
-    <t>roller mouse</t>
-  </si>
-  <si>
-    <t>10000 sh</t>
-  </si>
-  <si>
-    <t>apple,HP</t>
-  </si>
-  <si>
-    <t>prod-6</t>
-  </si>
-  <si>
-    <t>vendor 4</t>
-  </si>
-  <si>
-    <t>spoons</t>
-  </si>
-  <si>
-    <t>silver</t>
-  </si>
-  <si>
-    <t>300 sh</t>
-  </si>
-  <si>
-    <t>kentra</t>
-  </si>
-  <si>
-    <t>delivery_id</t>
-  </si>
-  <si>
-    <t>pck_id</t>
-  </si>
-  <si>
-    <t>delivery_status</t>
-  </si>
-  <si>
-    <t>employee_id</t>
-  </si>
-  <si>
-    <t>delivery-1</t>
-  </si>
-  <si>
-    <t>pck-a</t>
-  </si>
-  <si>
-    <t>shipped</t>
-  </si>
-  <si>
-    <t>delivery-2</t>
-  </si>
-  <si>
-    <t>pck-b</t>
-  </si>
-  <si>
-    <t>in transit</t>
-  </si>
-  <si>
-    <t>delivery-3</t>
-  </si>
-  <si>
-    <t>pck-c</t>
-  </si>
-  <si>
-    <t>in-transit</t>
-  </si>
-  <si>
-    <t>delivery-4</t>
-  </si>
-  <si>
-    <t>pck-d</t>
-  </si>
-  <si>
-    <t>station</t>
-  </si>
-  <si>
-    <t>delivery-5</t>
-  </si>
-  <si>
-    <t>pck-e</t>
-  </si>
-  <si>
-    <t>limuru station</t>
-  </si>
-  <si>
-    <t>limuru</t>
-  </si>
-  <si>
-    <t>nairobi</t>
-  </si>
-  <si>
-    <t>mombasa</t>
-  </si>
-  <si>
-    <t>kisumu</t>
-  </si>
-  <si>
-    <t>machakos</t>
-  </si>
-  <si>
-    <t>payment_id</t>
-  </si>
-  <si>
-    <t>payment method</t>
-  </si>
-  <si>
-    <t>payment status</t>
-  </si>
-  <si>
-    <t>payment-1</t>
-  </si>
-  <si>
-    <t>m-pesa</t>
-  </si>
-  <si>
-    <t>partial</t>
-  </si>
-  <si>
-    <t>payment-2</t>
-  </si>
-  <si>
-    <t>card</t>
-  </si>
-  <si>
-    <t>payment-3</t>
-  </si>
-  <si>
-    <t>mpesa</t>
-  </si>
-  <si>
-    <t>full</t>
-  </si>
-  <si>
-    <t>payment-4</t>
-  </si>
-  <si>
-    <t>payment-5</t>
-  </si>
-  <si>
-    <t>user-02</t>
-  </si>
-  <si>
-    <t>user-03</t>
-  </si>
-  <si>
-    <t>user-08</t>
-  </si>
-  <si>
-    <t>user-09</t>
   </si>
 </sst>
 </file>
@@ -1960,6 +1952,41 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelCol="4"/>
+  <cols>
+    <col min="1" max="1" width="12.4545454545455" customWidth="1"/>
+    <col min="2" max="2" width="15.9090909090909" customWidth="1"/>
+    <col min="3" max="3" width="11.8181818181818" customWidth="1"/>
+    <col min="4" max="4" width="9.81818181818182" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C1" t="s">
+        <v>144</v>
+      </c>
+      <c r="D1" t="s">
+        <v>145</v>
+      </c>
+      <c r="E1" t="s">
+        <v>146</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C6"/>
   <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="5" outlineLevelCol="2"/>
   <cols>
@@ -1970,233 +1997,53 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B3" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B4" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B6" t="s">
-        <v>158</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:G7"/>
-  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="6" outlineLevelCol="6"/>
-  <cols>
-    <col min="1" max="1" width="9.81818181818182" customWidth="1"/>
-    <col min="2" max="2" width="10.8181818181818" customWidth="1"/>
-    <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="17.3636363636364" customWidth="1"/>
-    <col min="7" max="7" width="21.3636363636364" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" t="s">
-        <v>135</v>
-      </c>
-      <c r="B1" t="s">
-        <v>146</v>
-      </c>
-      <c r="C1" t="s">
         <v>159</v>
-      </c>
-      <c r="D1" t="s">
-        <v>147</v>
-      </c>
-      <c r="E1" t="s">
-        <v>148</v>
-      </c>
-      <c r="F1" t="s">
-        <v>160</v>
-      </c>
-      <c r="G1" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" t="s">
-        <v>137</v>
-      </c>
-      <c r="B2" t="s">
-        <v>149</v>
-      </c>
-      <c r="C2" t="s">
-        <v>162</v>
-      </c>
-      <c r="D2" t="s">
-        <v>163</v>
-      </c>
-      <c r="E2" t="s">
-        <v>164</v>
-      </c>
-      <c r="F2" t="s">
-        <v>165</v>
-      </c>
-      <c r="G2" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" t="s">
-        <v>139</v>
-      </c>
-      <c r="B3" t="s">
-        <v>151</v>
-      </c>
-      <c r="C3" t="s">
-        <v>167</v>
-      </c>
-      <c r="D3" t="s">
-        <v>168</v>
-      </c>
-      <c r="E3" t="s">
-        <v>169</v>
-      </c>
-      <c r="F3" t="s">
-        <v>170</v>
-      </c>
-      <c r="G3" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" t="s">
-        <v>141</v>
-      </c>
-      <c r="B4" t="s">
-        <v>153</v>
-      </c>
-      <c r="C4" t="s">
-        <v>172</v>
-      </c>
-      <c r="D4" t="s">
-        <v>173</v>
-      </c>
-      <c r="E4" t="s">
-        <v>174</v>
-      </c>
-      <c r="F4" t="s">
-        <v>175</v>
-      </c>
-      <c r="G4" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" t="s">
-        <v>143</v>
-      </c>
-      <c r="B5" t="s">
-        <v>149</v>
-      </c>
-      <c r="C5" t="s">
-        <v>177</v>
-      </c>
-      <c r="D5" t="s">
-        <v>178</v>
-      </c>
-      <c r="E5" t="s">
-        <v>179</v>
-      </c>
-      <c r="F5" t="s">
-        <v>180</v>
-      </c>
-      <c r="G5" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" t="s">
-        <v>145</v>
-      </c>
-      <c r="B6" t="s">
-        <v>149</v>
-      </c>
-      <c r="C6" t="s">
-        <v>182</v>
-      </c>
-      <c r="D6" t="s">
-        <v>183</v>
-      </c>
-      <c r="E6" t="s">
-        <v>184</v>
-      </c>
-      <c r="F6" t="s">
-        <v>185</v>
-      </c>
-      <c r="G6" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" t="s">
-        <v>187</v>
-      </c>
-      <c r="B7" t="s">
-        <v>155</v>
-      </c>
-      <c r="C7" t="s">
-        <v>188</v>
-      </c>
-      <c r="D7" t="s">
-        <v>189</v>
-      </c>
-      <c r="E7" t="s">
-        <v>190</v>
-      </c>
-      <c r="F7" t="s">
-        <v>191</v>
-      </c>
-      <c r="G7" t="s">
-        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -2206,6 +2053,144 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="6" outlineLevelCol="4"/>
+  <cols>
+    <col min="1" max="1" width="9.81818181818182" customWidth="1"/>
+    <col min="2" max="2" width="10.8181818181818" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="17.3636363636364" customWidth="1"/>
+    <col min="5" max="5" width="21.3636363636364" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>144</v>
+      </c>
+      <c r="B1" t="s">
+        <v>147</v>
+      </c>
+      <c r="C1" t="s">
+        <v>148</v>
+      </c>
+      <c r="D1" t="s">
+        <v>149</v>
+      </c>
+      <c r="E1" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C2" t="s">
+        <v>162</v>
+      </c>
+      <c r="D2" t="s">
+        <v>163</v>
+      </c>
+      <c r="E2" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>165</v>
+      </c>
+      <c r="B3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C3" t="s">
+        <v>166</v>
+      </c>
+      <c r="D3" t="s">
+        <v>167</v>
+      </c>
+      <c r="E3" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>169</v>
+      </c>
+      <c r="B4" t="s">
+        <v>154</v>
+      </c>
+      <c r="C4" t="s">
+        <v>170</v>
+      </c>
+      <c r="D4" t="s">
+        <v>171</v>
+      </c>
+      <c r="E4" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>173</v>
+      </c>
+      <c r="B5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C5" t="s">
+        <v>174</v>
+      </c>
+      <c r="D5" t="s">
+        <v>175</v>
+      </c>
+      <c r="E5" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>177</v>
+      </c>
+      <c r="B6" t="s">
+        <v>150</v>
+      </c>
+      <c r="C6" t="s">
+        <v>178</v>
+      </c>
+      <c r="D6" t="s">
+        <v>179</v>
+      </c>
+      <c r="E6" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
+        <v>181</v>
+      </c>
+      <c r="B7" t="s">
+        <v>156</v>
+      </c>
+      <c r="C7" t="s">
+        <v>182</v>
+      </c>
+      <c r="D7" t="s">
+        <v>183</v>
+      </c>
+      <c r="E7" t="s">
+        <v>184</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:E6"/>
@@ -2219,33 +2204,33 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="B1" t="s">
         <v>120</v>
       </c>
       <c r="C1" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="D1" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="E1" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="B2" t="s">
         <v>123</v>
       </c>
       <c r="C2" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="D2" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="E2" t="s">
         <v>59</v>
@@ -2253,16 +2238,16 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="B3" t="s">
         <v>125</v>
       </c>
       <c r="C3" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="D3" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="E3" t="s">
         <v>59</v>
@@ -2270,16 +2255,16 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="B4" t="s">
         <v>127</v>
       </c>
       <c r="C4" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="D4" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="E4" t="s">
         <v>59</v>
@@ -2287,16 +2272,16 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="B5" t="s">
         <v>129</v>
       </c>
       <c r="C5" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="D5" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="E5" t="s">
         <v>59</v>
@@ -2304,16 +2289,16 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="B6" t="s">
         <v>131</v>
       </c>
       <c r="C6" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="D6" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="E6" t="s">
         <v>59</v>
@@ -2325,7 +2310,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:C6"/>
@@ -2336,68 +2321,68 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="B1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="B2" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="C2" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="B3" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="C3" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="B4" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="C4" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
+        <v>199</v>
+      </c>
+      <c r="B5" t="s">
         <v>207</v>
       </c>
-      <c r="B5" t="s">
-        <v>215</v>
-      </c>
       <c r="C5" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="B6" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="C6" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -2406,7 +2391,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:D6"/>
@@ -2420,86 +2405,86 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="B1" t="s">
         <v>120</v>
       </c>
       <c r="C1" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="D1" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="B2" t="s">
         <v>123</v>
       </c>
       <c r="C2" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="D2" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="B3" t="s">
         <v>125</v>
       </c>
       <c r="C3" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="D3" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="B4" t="s">
         <v>127</v>
       </c>
       <c r="C4" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="D4" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
       <c r="B5" t="s">
         <v>129</v>
       </c>
       <c r="C5" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="D5" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="B6" t="s">
         <v>131</v>
       </c>
       <c r="C6" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="D6" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
     </row>
   </sheetData>
@@ -2508,7 +2493,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:D6"/>
@@ -2519,7 +2504,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>159</v>
+        <v>143</v>
       </c>
       <c r="B1" t="s">
         <v>7</v>
@@ -2533,7 +2518,7 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>162</v>
+        <v>222</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
@@ -2542,12 +2527,12 @@
         <v>2</v>
       </c>
       <c r="D2" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>167</v>
+        <v>224</v>
       </c>
       <c r="B3" t="s">
         <v>11</v>
@@ -2556,12 +2541,12 @@
         <v>3</v>
       </c>
       <c r="D3" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>172</v>
+        <v>226</v>
       </c>
       <c r="B4" t="s">
         <v>13</v>
@@ -2570,12 +2555,12 @@
         <v>4</v>
       </c>
       <c r="D4" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>177</v>
+        <v>228</v>
       </c>
       <c r="B5" t="s">
         <v>15</v>
@@ -2584,12 +2569,12 @@
         <v>5</v>
       </c>
       <c r="D5" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>182</v>
+        <v>230</v>
       </c>
       <c r="B6" t="s">
         <v>17</v>
@@ -3441,15 +3426,15 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="5" outlineLevelCol="3"/>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="5" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="1" width="12.4545454545455" customWidth="1"/>
     <col min="2" max="2" width="15.9090909090909" customWidth="1"/>
     <col min="4" max="4" width="9.81818181818182" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>120</v>
       </c>
@@ -3462,8 +3447,17 @@
       <c r="D1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
+      <c r="E1" t="s">
+        <v>136</v>
+      </c>
+      <c r="F1" t="s">
+        <v>134</v>
+      </c>
+      <c r="G1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>123</v>
       </c>
@@ -3471,13 +3465,10 @@
         <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>136</v>
-      </c>
-      <c r="D2" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>125</v>
       </c>
@@ -3485,13 +3476,10 @@
         <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>138</v>
-      </c>
-      <c r="D3" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>127</v>
       </c>
@@ -3501,11 +3489,8 @@
       <c r="C4" t="s">
         <v>140</v>
       </c>
-      <c r="D4" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
+    </row>
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>129</v>
       </c>
@@ -3513,13 +3498,10 @@
         <v>13</v>
       </c>
       <c r="C5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D5" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>131</v>
       </c>
@@ -3527,10 +3509,7 @@
         <v>14</v>
       </c>
       <c r="C6" t="s">
-        <v>144</v>
-      </c>
-      <c r="D6" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>

</xml_diff>